<commit_message>
feat: atualizar formula de PnL para liability fixa =SE(L2=1; 0,965/(Odd_lay-1); -1)
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_Odds_Reais_Betfair.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_Odds_Reais_Betfair.xlsx
@@ -16,10 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -58,12 +55,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P190"/>
+  <dimension ref="A1:Q190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,10 +509,17 @@
           <t>PnL_u</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>P/L</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>46255</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -583,12 +586,17 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>0.955</v>
+        <v>0.1856</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.1856</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>46255</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -655,12 +663,17 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>0.955</v>
+        <v>0.1508</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.1508</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>46255</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -727,12 +740,17 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>0.955</v>
+        <v>0.1856</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.1856</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>46255</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -799,12 +817,17 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>0.955</v>
+        <v>0.1379</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.1379</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>46255</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -871,12 +894,17 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>0.955</v>
+        <v>0.201</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.201</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>46255</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -943,12 +971,17 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>0.955</v>
+        <v>0.1419</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0.1419</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>46255</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -1015,12 +1048,17 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>0.955</v>
+        <v>0.2144</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.2144</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>46255</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1087,12 +1125,17 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>0.955</v>
+        <v>0.193</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.193</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>46255</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1159,12 +1202,17 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>-5.8</v>
+        <v>-1</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>46255</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1231,12 +1279,17 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>0.955</v>
+        <v>0.1508</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0.1508</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>46255</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1303,12 +1356,17 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>0.955</v>
+        <v>0.1379</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0.1379</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>46256</v>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1375,12 +1433,17 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>0.955</v>
+        <v>0.2053</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0.2053</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>46256</v>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1447,12 +1510,17 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>0.955</v>
+        <v>0.1556</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0.1556</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>46256</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1519,12 +1587,17 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>0.955</v>
+        <v>0.201</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0.201</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>46256</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1591,12 +1664,17 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>-4.5</v>
+        <v>-1</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>46256</v>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1663,12 +1741,17 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>0.955</v>
+        <v>0.2053</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0.2053</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>46256</v>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1735,12 +1818,17 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>0.955</v>
+        <v>0.1237</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0.1237</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
-        <v>46256</v>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1807,12 +1895,17 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>0.955</v>
+        <v>0.1556</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0.1556</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
-        <v>46256</v>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1879,12 +1972,17 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>-5.4</v>
+        <v>-1</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
-        <v>46256</v>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1951,12 +2049,17 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>0.955</v>
+        <v>0.2193</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>0.2193</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>46256</v>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2023,12 +2126,17 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>0.955</v>
+        <v>0.1419</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0.1419</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
-        <v>46256</v>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2095,12 +2203,17 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>0.955</v>
+        <v>0.1856</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>0.1856</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>46256</v>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2167,12 +2280,17 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>0.955</v>
+        <v>0.1608</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0.1608</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
-        <v>46256</v>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2239,12 +2357,17 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>0.955</v>
+        <v>0.1723</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>0.1723</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
-        <v>46256</v>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2311,12 +2434,17 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>0.955</v>
+        <v>0.1856</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>0.1856</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n">
-        <v>46256</v>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2383,12 +2511,17 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>0.955</v>
+        <v>0.134</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>0.134</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
-        <v>46256</v>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2455,12 +2588,17 @@
         </is>
       </c>
       <c r="P28" t="n">
-        <v>0.955</v>
+        <v>0.1723</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>0.1723</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
-        <v>46256</v>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2527,12 +2665,17 @@
         </is>
       </c>
       <c r="P29" t="n">
-        <v>0.955</v>
+        <v>0.1664</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>0.1664</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
-        <v>46256</v>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2599,12 +2742,17 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>0.955</v>
+        <v>0.201</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>0.201</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
-        <v>46256</v>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2671,12 +2819,17 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>0.955</v>
+        <v>0.1787</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>0.1787</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
-        <v>46256</v>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2743,12 +2896,17 @@
         </is>
       </c>
       <c r="P32" t="n">
-        <v>0.955</v>
+        <v>0.134</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>0.134</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
-        <v>46256</v>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,12 +2973,17 @@
         </is>
       </c>
       <c r="P33" t="n">
-        <v>0.955</v>
+        <v>0.2053</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>0.2053</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
-        <v>46256</v>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2887,12 +3050,17 @@
         </is>
       </c>
       <c r="P34" t="n">
-        <v>0.955</v>
+        <v>0.1149</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>0.1149</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
-        <v>46256</v>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2959,12 +3127,17 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>-4.6</v>
+        <v>-1</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
-        <v>46256</v>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3031,12 +3204,17 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>0.955</v>
+        <v>0.127</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>0.127</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
-        <v>46256</v>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3103,12 +3281,17 @@
         </is>
       </c>
       <c r="P37" t="n">
-        <v>0.955</v>
+        <v>0.1608</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>0.1608</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
-        <v>46256</v>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3175,12 +3358,17 @@
         </is>
       </c>
       <c r="P38" t="n">
-        <v>0.955</v>
+        <v>0.0568</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>0.0568</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n">
-        <v>46256</v>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3247,12 +3435,17 @@
         </is>
       </c>
       <c r="P39" t="n">
-        <v>0.955</v>
+        <v>0.0536</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>0.0536</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
-        <v>46257</v>
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3319,12 +3512,17 @@
         </is>
       </c>
       <c r="P40" t="n">
-        <v>0.955</v>
+        <v>0.1723</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>0.1723</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
-        <v>46257</v>
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3391,12 +3589,17 @@
         </is>
       </c>
       <c r="P41" t="n">
-        <v>0.955</v>
+        <v>0.193</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>0.193</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
-        <v>46257</v>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3463,12 +3666,17 @@
         </is>
       </c>
       <c r="P42" t="n">
-        <v>0.955</v>
+        <v>0.1664</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>0.1664</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
-        <v>46257</v>
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3535,12 +3743,17 @@
         </is>
       </c>
       <c r="P43" t="n">
-        <v>0.955</v>
+        <v>0.1608</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>0.1608</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
-        <v>46257</v>
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3607,12 +3820,17 @@
         </is>
       </c>
       <c r="P44" t="n">
-        <v>0.955</v>
+        <v>0.1508</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>0.1508</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
-        <v>46257</v>
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -3679,12 +3897,17 @@
         </is>
       </c>
       <c r="P45" t="n">
-        <v>0.955</v>
+        <v>0.1608</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>0.1608</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
-        <v>46257</v>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -3751,12 +3974,17 @@
         </is>
       </c>
       <c r="P46" t="n">
-        <v>0.955</v>
+        <v>0.1462</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>0.1462</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n">
-        <v>46257</v>
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -3823,12 +4051,17 @@
         </is>
       </c>
       <c r="P47" t="n">
-        <v>0.955</v>
+        <v>0.1237</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>0.1237</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n">
-        <v>46257</v>
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -3895,12 +4128,17 @@
         </is>
       </c>
       <c r="P48" t="n">
-        <v>0.955</v>
+        <v>0.1379</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>0.1379</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n">
-        <v>46257</v>
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -3967,12 +4205,17 @@
         </is>
       </c>
       <c r="P49" t="n">
-        <v>0.955</v>
+        <v>0.1664</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>0.1664</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
-        <v>46257</v>
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -4039,12 +4282,17 @@
         </is>
       </c>
       <c r="P50" t="n">
-        <v>0.955</v>
+        <v>0.1723</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>0.1723</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n">
-        <v>46257</v>
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -4111,12 +4359,17 @@
         </is>
       </c>
       <c r="P51" t="n">
-        <v>0.955</v>
+        <v>0.1856</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>0.1856</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n">
-        <v>46257</v>
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -4183,12 +4436,17 @@
         </is>
       </c>
       <c r="P52" t="n">
-        <v>0.955</v>
+        <v>0.1664</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>0.1664</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n">
-        <v>46257</v>
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -4255,12 +4513,17 @@
         </is>
       </c>
       <c r="P53" t="n">
-        <v>-6</v>
+        <v>-1</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n">
-        <v>46257</v>
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -4327,12 +4590,17 @@
         </is>
       </c>
       <c r="P54" t="n">
-        <v>0.955</v>
+        <v>0.2053</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>0.2053</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n">
-        <v>46257</v>
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -4399,12 +4667,17 @@
         </is>
       </c>
       <c r="P55" t="n">
-        <v>0.955</v>
+        <v>0.1556</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>0.1556</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n">
-        <v>46257</v>
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -4471,12 +4744,17 @@
         </is>
       </c>
       <c r="P56" t="n">
-        <v>0.955</v>
+        <v>0.1304</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>0.1304</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n">
-        <v>46257</v>
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -4543,12 +4821,17 @@
         </is>
       </c>
       <c r="P57" t="n">
-        <v>0.955</v>
+        <v>0.127</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>0.127</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n">
-        <v>46257</v>
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -4615,12 +4898,17 @@
         </is>
       </c>
       <c r="P58" t="n">
-        <v>0.955</v>
+        <v>0.1608</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>0.1608</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n">
-        <v>46257</v>
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -4687,12 +4975,17 @@
         </is>
       </c>
       <c r="P59" t="n">
-        <v>0.955</v>
+        <v>0.1379</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>0.1379</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n">
-        <v>46257</v>
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -4759,12 +5052,17 @@
         </is>
       </c>
       <c r="P60" t="n">
-        <v>0.955</v>
+        <v>0.1122</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>0.1122</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n">
-        <v>46257</v>
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -4831,12 +5129,17 @@
         </is>
       </c>
       <c r="P61" t="n">
-        <v>0.955</v>
+        <v>0.1787</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>0.1787</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n">
-        <v>46257</v>
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -4903,12 +5206,17 @@
         </is>
       </c>
       <c r="P62" t="n">
-        <v>0.955</v>
+        <v>0.0568</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>0.0568</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n">
-        <v>46258</v>
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -4975,12 +5283,17 @@
         </is>
       </c>
       <c r="P63" t="n">
-        <v>0.955</v>
+        <v>0.2193</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>0.2193</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n">
-        <v>46258</v>
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -5047,12 +5360,17 @@
         </is>
       </c>
       <c r="P64" t="n">
-        <v>0.955</v>
+        <v>0.2193</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>0.2193</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n">
-        <v>46258</v>
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -5119,12 +5437,17 @@
         </is>
       </c>
       <c r="P65" t="n">
-        <v>0.955</v>
+        <v>0.1608</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>0.1608</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n">
-        <v>46258</v>
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -5191,12 +5514,17 @@
         </is>
       </c>
       <c r="P66" t="n">
-        <v>0.955</v>
+        <v>0.1664</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>0.1664</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n">
-        <v>46259</v>
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -5263,12 +5591,17 @@
         </is>
       </c>
       <c r="P67" t="n">
-        <v>0.955</v>
+        <v>0.2193</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>0.2193</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n">
-        <v>46259</v>
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -5335,12 +5668,17 @@
         </is>
       </c>
       <c r="P68" t="n">
-        <v>0.955</v>
+        <v>0.1462</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>0.1462</v>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n">
-        <v>46259</v>
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -5407,12 +5745,17 @@
         </is>
       </c>
       <c r="P69" t="n">
-        <v>0.955</v>
+        <v>0.1206</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>0.1206</v>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="n">
-        <v>46259</v>
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -5479,12 +5822,17 @@
         </is>
       </c>
       <c r="P70" t="n">
-        <v>0.955</v>
+        <v>0.1856</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>0.1856</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="n">
-        <v>46259</v>
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -5551,12 +5899,17 @@
         </is>
       </c>
       <c r="P71" t="n">
-        <v>0.955</v>
+        <v>0.1723</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>0.1723</v>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n">
-        <v>46259</v>
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -5623,12 +5976,17 @@
         </is>
       </c>
       <c r="P72" t="n">
-        <v>0.955</v>
+        <v>0.0551</v>
+      </c>
+      <c r="Q72" t="n">
+        <v>0.0551</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="n">
-        <v>46259</v>
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -5691,10 +6049,15 @@
       <c r="P73" t="n">
         <v>0</v>
       </c>
+      <c r="Q73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="n">
-        <v>46260</v>
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -5761,12 +6124,17 @@
         </is>
       </c>
       <c r="P74" t="n">
-        <v>0.955</v>
+        <v>0.134</v>
+      </c>
+      <c r="Q74" t="n">
+        <v>0.134</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="n">
-        <v>46260</v>
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -5833,12 +6201,17 @@
         </is>
       </c>
       <c r="P75" t="n">
-        <v>0.955</v>
+        <v>0.1787</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>0.1787</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n">
-        <v>46260</v>
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
@@ -5905,12 +6278,17 @@
         </is>
       </c>
       <c r="P76" t="n">
-        <v>0.955</v>
+        <v>0.193</v>
+      </c>
+      <c r="Q76" t="n">
+        <v>0.193</v>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="n">
-        <v>46260</v>
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
@@ -5977,12 +6355,17 @@
         </is>
       </c>
       <c r="P77" t="n">
-        <v>0.955</v>
+        <v>0.1608</v>
+      </c>
+      <c r="Q77" t="n">
+        <v>0.1608</v>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n">
-        <v>46260</v>
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
@@ -6049,12 +6432,17 @@
         </is>
       </c>
       <c r="P78" t="n">
-        <v>0.955</v>
+        <v>0.1664</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>0.1664</v>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="n">
-        <v>46260</v>
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -6121,12 +6509,17 @@
         </is>
       </c>
       <c r="P79" t="n">
-        <v>0.955</v>
+        <v>0.1969</v>
+      </c>
+      <c r="Q79" t="n">
+        <v>0.1969</v>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="n">
-        <v>46260</v>
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -6189,10 +6582,15 @@
       <c r="P80" t="n">
         <v>0</v>
       </c>
+      <c r="Q80" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="n">
-        <v>46260</v>
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -6259,12 +6657,17 @@
         </is>
       </c>
       <c r="P81" t="n">
-        <v>-6.2</v>
+        <v>-1</v>
+      </c>
+      <c r="Q81" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n">
-        <v>46260</v>
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -6331,12 +6734,17 @@
         </is>
       </c>
       <c r="P82" t="n">
-        <v>-4.2</v>
+        <v>-1</v>
+      </c>
+      <c r="Q82" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="n">
-        <v>46260</v>
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
@@ -6403,12 +6811,17 @@
         </is>
       </c>
       <c r="P83" t="n">
-        <v>0.955</v>
+        <v>0.1556</v>
+      </c>
+      <c r="Q83" t="n">
+        <v>0.1556</v>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n">
-        <v>46260</v>
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -6475,12 +6888,17 @@
         </is>
       </c>
       <c r="P84" t="n">
-        <v>0.955</v>
+        <v>0.0522</v>
+      </c>
+      <c r="Q84" t="n">
+        <v>0.0522</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="n">
-        <v>46261</v>
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
@@ -6547,12 +6965,17 @@
         </is>
       </c>
       <c r="P85" t="n">
-        <v>0.955</v>
+        <v>0.1177</v>
+      </c>
+      <c r="Q85" t="n">
+        <v>0.1177</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n">
-        <v>46261</v>
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
@@ -6619,12 +7042,17 @@
         </is>
       </c>
       <c r="P86" t="n">
-        <v>0.955</v>
+        <v>0.1787</v>
+      </c>
+      <c r="Q86" t="n">
+        <v>0.1787</v>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="n">
-        <v>46261</v>
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
@@ -6691,12 +7119,17 @@
         </is>
       </c>
       <c r="P87" t="n">
-        <v>0.955</v>
+        <v>0.1856</v>
+      </c>
+      <c r="Q87" t="n">
+        <v>0.1856</v>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="n">
-        <v>46261</v>
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -6763,12 +7196,17 @@
         </is>
       </c>
       <c r="P88" t="n">
-        <v>0.955</v>
+        <v>0.2193</v>
+      </c>
+      <c r="Q88" t="n">
+        <v>0.2193</v>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="n">
-        <v>46261</v>
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
@@ -6835,12 +7273,17 @@
         </is>
       </c>
       <c r="P89" t="n">
-        <v>0.955</v>
+        <v>0.1462</v>
+      </c>
+      <c r="Q89" t="n">
+        <v>0.1462</v>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n">
-        <v>46261</v>
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
@@ -6907,12 +7350,17 @@
         </is>
       </c>
       <c r="P90" t="n">
-        <v>0.955</v>
+        <v>0.1723</v>
+      </c>
+      <c r="Q90" t="n">
+        <v>0.1723</v>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="n">
-        <v>46261</v>
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
@@ -6979,12 +7427,17 @@
         </is>
       </c>
       <c r="P91" t="n">
-        <v>0.955</v>
+        <v>0.1072</v>
+      </c>
+      <c r="Q91" t="n">
+        <v>0.1072</v>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="n">
-        <v>46261</v>
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
@@ -7051,12 +7504,17 @@
         </is>
       </c>
       <c r="P92" t="n">
-        <v>0.955</v>
+        <v>0.1462</v>
+      </c>
+      <c r="Q92" t="n">
+        <v>0.1462</v>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="n">
-        <v>46261</v>
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
@@ -7123,12 +7581,17 @@
         </is>
       </c>
       <c r="P93" t="n">
-        <v>0.955</v>
+        <v>0.2098</v>
+      </c>
+      <c r="Q93" t="n">
+        <v>0.2098</v>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="n">
-        <v>46261</v>
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
@@ -7195,12 +7658,17 @@
         </is>
       </c>
       <c r="P94" t="n">
-        <v>-6.2</v>
+        <v>-1</v>
+      </c>
+      <c r="Q94" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="2" t="n">
-        <v>46261</v>
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
@@ -7267,12 +7735,17 @@
         </is>
       </c>
       <c r="P95" t="n">
-        <v>0.955</v>
+        <v>0.1419</v>
+      </c>
+      <c r="Q95" t="n">
+        <v>0.1419</v>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="n">
-        <v>46261</v>
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
@@ -7339,12 +7812,17 @@
         </is>
       </c>
       <c r="P96" t="n">
-        <v>0.955</v>
+        <v>0.1419</v>
+      </c>
+      <c r="Q96" t="n">
+        <v>0.1419</v>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="2" t="n">
-        <v>46261</v>
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
@@ -7411,12 +7889,17 @@
         </is>
       </c>
       <c r="P97" t="n">
-        <v>-9</v>
+        <v>-1</v>
+      </c>
+      <c r="Q97" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="n">
-        <v>46261</v>
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -7483,12 +7966,17 @@
         </is>
       </c>
       <c r="P98" t="n">
-        <v>0.955</v>
+        <v>0.1462</v>
+      </c>
+      <c r="Q98" t="n">
+        <v>0.1462</v>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="n">
-        <v>46261</v>
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
@@ -7555,12 +8043,17 @@
         </is>
       </c>
       <c r="P99" t="n">
-        <v>0.955</v>
+        <v>0.1379</v>
+      </c>
+      <c r="Q99" t="n">
+        <v>0.1379</v>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="n">
-        <v>46261</v>
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
@@ -7627,12 +8120,17 @@
         </is>
       </c>
       <c r="P100" t="n">
-        <v>0.955</v>
+        <v>0.1072</v>
+      </c>
+      <c r="Q100" t="n">
+        <v>0.1072</v>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="n">
-        <v>46261</v>
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
@@ -7699,12 +8197,17 @@
         </is>
       </c>
       <c r="P101" t="n">
-        <v>0.955</v>
+        <v>0.0568</v>
+      </c>
+      <c r="Q101" t="n">
+        <v>0.0568</v>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="n">
-        <v>46262</v>
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
@@ -7771,12 +8274,17 @@
         </is>
       </c>
       <c r="P102" t="n">
-        <v>0.955</v>
+        <v>0.1723</v>
+      </c>
+      <c r="Q102" t="n">
+        <v>0.1723</v>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="n">
-        <v>46262</v>
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -7843,12 +8351,17 @@
         </is>
       </c>
       <c r="P103" t="n">
-        <v>0.955</v>
+        <v>0.1664</v>
+      </c>
+      <c r="Q103" t="n">
+        <v>0.1664</v>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="n">
-        <v>46262</v>
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -7915,12 +8428,17 @@
         </is>
       </c>
       <c r="P104" t="n">
-        <v>0.955</v>
+        <v>0.1304</v>
+      </c>
+      <c r="Q104" t="n">
+        <v>0.1304</v>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="n">
-        <v>46262</v>
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
@@ -7987,12 +8505,17 @@
         </is>
       </c>
       <c r="P105" t="n">
-        <v>0.955</v>
+        <v>0.1723</v>
+      </c>
+      <c r="Q105" t="n">
+        <v>0.1723</v>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="n">
-        <v>46262</v>
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
@@ -8059,12 +8582,17 @@
         </is>
       </c>
       <c r="P106" t="n">
-        <v>0.955</v>
+        <v>0.1379</v>
+      </c>
+      <c r="Q106" t="n">
+        <v>0.1379</v>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="n">
-        <v>46262</v>
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
@@ -8131,12 +8659,17 @@
         </is>
       </c>
       <c r="P107" t="n">
-        <v>0.955</v>
+        <v>0.1664</v>
+      </c>
+      <c r="Q107" t="n">
+        <v>0.1664</v>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="n">
-        <v>46262</v>
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
@@ -8203,12 +8736,17 @@
         </is>
       </c>
       <c r="P108" t="n">
-        <v>0.955</v>
+        <v>0.2053</v>
+      </c>
+      <c r="Q108" t="n">
+        <v>0.2053</v>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="2" t="n">
-        <v>46262</v>
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
@@ -8275,12 +8813,17 @@
         </is>
       </c>
       <c r="P109" t="n">
-        <v>0.955</v>
+        <v>0.127</v>
+      </c>
+      <c r="Q109" t="n">
+        <v>0.127</v>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="2" t="n">
-        <v>46262</v>
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
@@ -8347,12 +8890,17 @@
         </is>
       </c>
       <c r="P110" t="n">
-        <v>0.955</v>
+        <v>0.1608</v>
+      </c>
+      <c r="Q110" t="n">
+        <v>0.1608</v>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="n">
-        <v>46262</v>
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
@@ -8419,12 +8967,17 @@
         </is>
       </c>
       <c r="P111" t="n">
-        <v>0.955</v>
+        <v>0.1664</v>
+      </c>
+      <c r="Q111" t="n">
+        <v>0.1664</v>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="n">
-        <v>46262</v>
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
@@ -8491,12 +9044,17 @@
         </is>
       </c>
       <c r="P112" t="n">
-        <v>0.955</v>
+        <v>0.201</v>
+      </c>
+      <c r="Q112" t="n">
+        <v>0.201</v>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="2" t="n">
-        <v>46262</v>
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
@@ -8563,12 +9121,17 @@
         </is>
       </c>
       <c r="P113" t="n">
-        <v>0.955</v>
+        <v>0.134</v>
+      </c>
+      <c r="Q113" t="n">
+        <v>0.134</v>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="n">
-        <v>46262</v>
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
@@ -8635,12 +9198,17 @@
         </is>
       </c>
       <c r="P114" t="n">
-        <v>0.955</v>
+        <v>0.1664</v>
+      </c>
+      <c r="Q114" t="n">
+        <v>0.1664</v>
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="2" t="n">
-        <v>46262</v>
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
@@ -8707,12 +9275,17 @@
         </is>
       </c>
       <c r="P115" t="n">
-        <v>0.955</v>
+        <v>0.0508</v>
+      </c>
+      <c r="Q115" t="n">
+        <v>0.0508</v>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="2" t="n">
-        <v>46263</v>
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
@@ -8779,12 +9352,17 @@
         </is>
       </c>
       <c r="P116" t="n">
-        <v>0.955</v>
+        <v>0.1608</v>
+      </c>
+      <c r="Q116" t="n">
+        <v>0.1608</v>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="2" t="n">
-        <v>46263</v>
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
@@ -8851,12 +9429,17 @@
         </is>
       </c>
       <c r="P117" t="n">
-        <v>0.955</v>
+        <v>0.1856</v>
+      </c>
+      <c r="Q117" t="n">
+        <v>0.1856</v>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="2" t="n">
-        <v>46263</v>
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
@@ -8923,12 +9506,17 @@
         </is>
       </c>
       <c r="P118" t="n">
-        <v>0.955</v>
+        <v>0.1097</v>
+      </c>
+      <c r="Q118" t="n">
+        <v>0.1097</v>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="2" t="n">
-        <v>46263</v>
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
@@ -8995,12 +9583,17 @@
         </is>
       </c>
       <c r="P119" t="n">
-        <v>-4.9</v>
+        <v>-1</v>
+      </c>
+      <c r="Q119" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="2" t="n">
-        <v>46263</v>
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
@@ -9067,12 +9660,17 @@
         </is>
       </c>
       <c r="P120" t="n">
-        <v>0.955</v>
+        <v>0.1608</v>
+      </c>
+      <c r="Q120" t="n">
+        <v>0.1608</v>
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="2" t="n">
-        <v>46263</v>
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
@@ -9139,12 +9737,17 @@
         </is>
       </c>
       <c r="P121" t="n">
-        <v>0.955</v>
+        <v>0.193</v>
+      </c>
+      <c r="Q121" t="n">
+        <v>0.193</v>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="2" t="n">
-        <v>46263</v>
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
@@ -9211,12 +9814,17 @@
         </is>
       </c>
       <c r="P122" t="n">
-        <v>0.955</v>
+        <v>0.1787</v>
+      </c>
+      <c r="Q122" t="n">
+        <v>0.1787</v>
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="2" t="n">
-        <v>46263</v>
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
@@ -9283,12 +9891,17 @@
         </is>
       </c>
       <c r="P123" t="n">
-        <v>0.955</v>
+        <v>0.1787</v>
+      </c>
+      <c r="Q123" t="n">
+        <v>0.1787</v>
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="2" t="n">
-        <v>46263</v>
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -9355,12 +9968,17 @@
         </is>
       </c>
       <c r="P124" t="n">
-        <v>0.955</v>
+        <v>0.1664</v>
+      </c>
+      <c r="Q124" t="n">
+        <v>0.1664</v>
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="2" t="n">
-        <v>46263</v>
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -9427,12 +10045,17 @@
         </is>
       </c>
       <c r="P125" t="n">
-        <v>0.955</v>
+        <v>0.1664</v>
+      </c>
+      <c r="Q125" t="n">
+        <v>0.1664</v>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="2" t="n">
-        <v>46263</v>
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -9499,12 +10122,17 @@
         </is>
       </c>
       <c r="P126" t="n">
-        <v>0.955</v>
+        <v>0.1664</v>
+      </c>
+      <c r="Q126" t="n">
+        <v>0.1664</v>
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="2" t="n">
-        <v>46263</v>
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -9571,12 +10199,17 @@
         </is>
       </c>
       <c r="P127" t="n">
-        <v>0.955</v>
+        <v>0.2144</v>
+      </c>
+      <c r="Q127" t="n">
+        <v>0.2144</v>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="2" t="n">
-        <v>46263</v>
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
@@ -9643,12 +10276,17 @@
         </is>
       </c>
       <c r="P128" t="n">
-        <v>0.955</v>
+        <v>0.1856</v>
+      </c>
+      <c r="Q128" t="n">
+        <v>0.1856</v>
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="2" t="n">
-        <v>46263</v>
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -9715,12 +10353,17 @@
         </is>
       </c>
       <c r="P129" t="n">
-        <v>0.955</v>
+        <v>0.201</v>
+      </c>
+      <c r="Q129" t="n">
+        <v>0.201</v>
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="2" t="n">
-        <v>46263</v>
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
@@ -9787,12 +10430,17 @@
         </is>
       </c>
       <c r="P130" t="n">
-        <v>0.955</v>
+        <v>0.1206</v>
+      </c>
+      <c r="Q130" t="n">
+        <v>0.1206</v>
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="2" t="n">
-        <v>46263</v>
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
@@ -9859,12 +10507,17 @@
         </is>
       </c>
       <c r="P131" t="n">
-        <v>0.955</v>
+        <v>0.1379</v>
+      </c>
+      <c r="Q131" t="n">
+        <v>0.1379</v>
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="2" t="n">
-        <v>46263</v>
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
@@ -9931,12 +10584,17 @@
         </is>
       </c>
       <c r="P132" t="n">
-        <v>0.955</v>
+        <v>0.1304</v>
+      </c>
+      <c r="Q132" t="n">
+        <v>0.1304</v>
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="2" t="n">
-        <v>46263</v>
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
@@ -10003,12 +10661,17 @@
         </is>
       </c>
       <c r="P133" t="n">
-        <v>0.955</v>
+        <v>0.1462</v>
+      </c>
+      <c r="Q133" t="n">
+        <v>0.1462</v>
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="2" t="n">
-        <v>46263</v>
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
@@ -10075,12 +10738,17 @@
         </is>
       </c>
       <c r="P134" t="n">
-        <v>0.955</v>
+        <v>0.0568</v>
+      </c>
+      <c r="Q134" t="n">
+        <v>0.0568</v>
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="2" t="n">
-        <v>46263</v>
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
@@ -10147,12 +10815,17 @@
         </is>
       </c>
       <c r="P135" t="n">
-        <v>0.955</v>
+        <v>0.1016</v>
+      </c>
+      <c r="Q135" t="n">
+        <v>0.1016</v>
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="2" t="n">
-        <v>46263</v>
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -10219,12 +10892,17 @@
         </is>
       </c>
       <c r="P136" t="n">
-        <v>0.955</v>
+        <v>0.0551</v>
+      </c>
+      <c r="Q136" t="n">
+        <v>0.0551</v>
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="2" t="n">
-        <v>46264</v>
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
@@ -10291,12 +10969,17 @@
         </is>
       </c>
       <c r="P137" t="n">
-        <v>0.955</v>
+        <v>0.193</v>
+      </c>
+      <c r="Q137" t="n">
+        <v>0.193</v>
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="2" t="n">
-        <v>46264</v>
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
@@ -10363,12 +11046,17 @@
         </is>
       </c>
       <c r="P138" t="n">
-        <v>-8.199999999999999</v>
+        <v>-1</v>
+      </c>
+      <c r="Q138" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="2" t="n">
-        <v>46264</v>
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
@@ -10435,12 +11123,17 @@
         </is>
       </c>
       <c r="P139" t="n">
-        <v>0.955</v>
+        <v>0.1664</v>
+      </c>
+      <c r="Q139" t="n">
+        <v>0.1664</v>
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="2" t="n">
-        <v>46264</v>
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
@@ -10507,12 +11200,17 @@
         </is>
       </c>
       <c r="P140" t="n">
-        <v>0.955</v>
+        <v>0.193</v>
+      </c>
+      <c r="Q140" t="n">
+        <v>0.193</v>
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="2" t="n">
-        <v>46264</v>
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
@@ -10579,12 +11277,17 @@
         </is>
       </c>
       <c r="P141" t="n">
-        <v>0.955</v>
+        <v>0.1664</v>
+      </c>
+      <c r="Q141" t="n">
+        <v>0.1664</v>
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="2" t="n">
-        <v>46264</v>
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
@@ -10651,12 +11354,17 @@
         </is>
       </c>
       <c r="P142" t="n">
-        <v>0.955</v>
+        <v>0.1608</v>
+      </c>
+      <c r="Q142" t="n">
+        <v>0.1608</v>
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="2" t="n">
-        <v>46264</v>
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
@@ -10723,12 +11431,17 @@
         </is>
       </c>
       <c r="P143" t="n">
-        <v>0.955</v>
+        <v>0.201</v>
+      </c>
+      <c r="Q143" t="n">
+        <v>0.201</v>
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="2" t="n">
-        <v>46264</v>
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
@@ -10795,12 +11508,17 @@
         </is>
       </c>
       <c r="P144" t="n">
-        <v>0.955</v>
+        <v>0.1969</v>
+      </c>
+      <c r="Q144" t="n">
+        <v>0.1969</v>
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="2" t="n">
-        <v>46264</v>
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
@@ -10867,12 +11585,17 @@
         </is>
       </c>
       <c r="P145" t="n">
-        <v>0.955</v>
+        <v>0.1723</v>
+      </c>
+      <c r="Q145" t="n">
+        <v>0.1723</v>
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="2" t="n">
-        <v>46264</v>
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
@@ -10939,12 +11662,17 @@
         </is>
       </c>
       <c r="P146" t="n">
-        <v>0.955</v>
+        <v>0.1723</v>
+      </c>
+      <c r="Q146" t="n">
+        <v>0.1723</v>
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="2" t="n">
-        <v>46264</v>
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
@@ -11011,12 +11739,17 @@
         </is>
       </c>
       <c r="P147" t="n">
-        <v>-4.7</v>
+        <v>-1</v>
+      </c>
+      <c r="Q147" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="2" t="n">
-        <v>46264</v>
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
@@ -11083,12 +11816,17 @@
         </is>
       </c>
       <c r="P148" t="n">
-        <v>0.955</v>
+        <v>0.1097</v>
+      </c>
+      <c r="Q148" t="n">
+        <v>0.1097</v>
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="2" t="n">
-        <v>46264</v>
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
@@ -11155,12 +11893,17 @@
         </is>
       </c>
       <c r="P149" t="n">
-        <v>-5.4</v>
+        <v>-1</v>
+      </c>
+      <c r="Q149" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="2" t="n">
-        <v>46264</v>
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
@@ -11227,12 +11970,17 @@
         </is>
       </c>
       <c r="P150" t="n">
-        <v>0.955</v>
+        <v>0.201</v>
+      </c>
+      <c r="Q150" t="n">
+        <v>0.201</v>
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="2" t="n">
-        <v>46264</v>
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
@@ -11299,12 +12047,17 @@
         </is>
       </c>
       <c r="P151" t="n">
-        <v>0.955</v>
+        <v>0.1177</v>
+      </c>
+      <c r="Q151" t="n">
+        <v>0.1177</v>
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="2" t="n">
-        <v>46264</v>
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
@@ -11371,12 +12124,17 @@
         </is>
       </c>
       <c r="P152" t="n">
-        <v>-4.6</v>
+        <v>-1</v>
+      </c>
+      <c r="Q152" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="2" t="n">
-        <v>46264</v>
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
@@ -11443,12 +12201,17 @@
         </is>
       </c>
       <c r="P153" t="n">
-        <v>0.955</v>
+        <v>0.1723</v>
+      </c>
+      <c r="Q153" t="n">
+        <v>0.1723</v>
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="2" t="n">
-        <v>46264</v>
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
@@ -11515,12 +12278,17 @@
         </is>
       </c>
       <c r="P154" t="n">
-        <v>0.955</v>
+        <v>0.201</v>
+      </c>
+      <c r="Q154" t="n">
+        <v>0.201</v>
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="2" t="n">
-        <v>46264</v>
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
@@ -11587,12 +12355,17 @@
         </is>
       </c>
       <c r="P155" t="n">
-        <v>0.955</v>
+        <v>0.1379</v>
+      </c>
+      <c r="Q155" t="n">
+        <v>0.1379</v>
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="2" t="n">
-        <v>46264</v>
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
@@ -11659,12 +12432,17 @@
         </is>
       </c>
       <c r="P156" t="n">
-        <v>0.955</v>
+        <v>0.1508</v>
+      </c>
+      <c r="Q156" t="n">
+        <v>0.1508</v>
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="2" t="n">
-        <v>46264</v>
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
@@ -11731,12 +12509,17 @@
         </is>
       </c>
       <c r="P157" t="n">
-        <v>0.955</v>
+        <v>0.1664</v>
+      </c>
+      <c r="Q157" t="n">
+        <v>0.1664</v>
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="2" t="n">
-        <v>46264</v>
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
@@ -11803,12 +12586,17 @@
         </is>
       </c>
       <c r="P158" t="n">
-        <v>0.955</v>
+        <v>0.1664</v>
+      </c>
+      <c r="Q158" t="n">
+        <v>0.1664</v>
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="2" t="n">
-        <v>46264</v>
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
@@ -11875,12 +12663,17 @@
         </is>
       </c>
       <c r="P159" t="n">
-        <v>0.955</v>
+        <v>0.1787</v>
+      </c>
+      <c r="Q159" t="n">
+        <v>0.1787</v>
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="2" t="n">
-        <v>46264</v>
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
@@ -11947,12 +12740,17 @@
         </is>
       </c>
       <c r="P160" t="n">
-        <v>0.955</v>
+        <v>0.2053</v>
+      </c>
+      <c r="Q160" t="n">
+        <v>0.2053</v>
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="2" t="n">
-        <v>46264</v>
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
@@ -12019,12 +12817,17 @@
         </is>
       </c>
       <c r="P161" t="n">
-        <v>0.955</v>
+        <v>0.2298</v>
+      </c>
+      <c r="Q161" t="n">
+        <v>0.2298</v>
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="2" t="n">
-        <v>46264</v>
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
@@ -12091,12 +12894,17 @@
         </is>
       </c>
       <c r="P162" t="n">
-        <v>0.955</v>
+        <v>0.1664</v>
+      </c>
+      <c r="Q162" t="n">
+        <v>0.1664</v>
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="2" t="n">
-        <v>46264</v>
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
@@ -12163,12 +12971,17 @@
         </is>
       </c>
       <c r="P163" t="n">
-        <v>0.955</v>
+        <v>0.1608</v>
+      </c>
+      <c r="Q163" t="n">
+        <v>0.1608</v>
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="2" t="n">
-        <v>46264</v>
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
@@ -12235,12 +13048,17 @@
         </is>
       </c>
       <c r="P164" t="n">
-        <v>0.955</v>
+        <v>0.1856</v>
+      </c>
+      <c r="Q164" t="n">
+        <v>0.1856</v>
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="2" t="n">
-        <v>46264</v>
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
@@ -12307,12 +13125,17 @@
         </is>
       </c>
       <c r="P165" t="n">
-        <v>0.955</v>
+        <v>0.1462</v>
+      </c>
+      <c r="Q165" t="n">
+        <v>0.1462</v>
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="2" t="n">
-        <v>46264</v>
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
@@ -12379,12 +13202,17 @@
         </is>
       </c>
       <c r="P166" t="n">
-        <v>0.955</v>
+        <v>0.1149</v>
+      </c>
+      <c r="Q166" t="n">
+        <v>0.1149</v>
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="2" t="n">
-        <v>46264</v>
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
@@ -12451,12 +13279,17 @@
         </is>
       </c>
       <c r="P167" t="n">
-        <v>0.955</v>
+        <v>0.1379</v>
+      </c>
+      <c r="Q167" t="n">
+        <v>0.1379</v>
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="2" t="n">
-        <v>46264</v>
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
@@ -12523,12 +13356,17 @@
         </is>
       </c>
       <c r="P168" t="n">
-        <v>0.955</v>
+        <v>0.1723</v>
+      </c>
+      <c r="Q168" t="n">
+        <v>0.1723</v>
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="2" t="n">
-        <v>46264</v>
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
@@ -12595,12 +13433,17 @@
         </is>
       </c>
       <c r="P169" t="n">
-        <v>0.955</v>
+        <v>0.1122</v>
+      </c>
+      <c r="Q169" t="n">
+        <v>0.1122</v>
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="2" t="n">
-        <v>46265</v>
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
@@ -12667,12 +13510,17 @@
         </is>
       </c>
       <c r="P170" t="n">
-        <v>-8</v>
+        <v>-1</v>
+      </c>
+      <c r="Q170" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="2" t="n">
-        <v>46265</v>
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
@@ -12739,12 +13587,17 @@
         </is>
       </c>
       <c r="P171" t="n">
-        <v>0.955</v>
+        <v>0.193</v>
+      </c>
+      <c r="Q171" t="n">
+        <v>0.193</v>
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="2" t="n">
-        <v>46265</v>
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
@@ -12811,12 +13664,17 @@
         </is>
       </c>
       <c r="P172" t="n">
-        <v>0.955</v>
+        <v>0.2144</v>
+      </c>
+      <c r="Q172" t="n">
+        <v>0.2144</v>
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="2" t="n">
-        <v>46265</v>
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
@@ -12883,12 +13741,17 @@
         </is>
       </c>
       <c r="P173" t="n">
-        <v>0.955</v>
+        <v>0.193</v>
+      </c>
+      <c r="Q173" t="n">
+        <v>0.193</v>
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="2" t="n">
-        <v>46265</v>
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
@@ -12955,12 +13818,17 @@
         </is>
       </c>
       <c r="P174" t="n">
-        <v>0.955</v>
+        <v>0.1419</v>
+      </c>
+      <c r="Q174" t="n">
+        <v>0.1419</v>
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="2" t="n">
-        <v>46265</v>
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
@@ -13027,12 +13895,17 @@
         </is>
       </c>
       <c r="P175" t="n">
-        <v>0.955</v>
+        <v>0.1608</v>
+      </c>
+      <c r="Q175" t="n">
+        <v>0.1608</v>
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="2" t="n">
-        <v>46265</v>
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
@@ -13099,12 +13972,17 @@
         </is>
       </c>
       <c r="P176" t="n">
-        <v>0.955</v>
+        <v>0.1723</v>
+      </c>
+      <c r="Q176" t="n">
+        <v>0.1723</v>
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="2" t="n">
-        <v>46265</v>
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
@@ -13171,12 +14049,17 @@
         </is>
       </c>
       <c r="P177" t="n">
-        <v>0.955</v>
+        <v>0.1304</v>
+      </c>
+      <c r="Q177" t="n">
+        <v>0.1304</v>
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="2" t="n">
-        <v>46265</v>
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
@@ -13243,12 +14126,17 @@
         </is>
       </c>
       <c r="P178" t="n">
-        <v>0.955</v>
+        <v>0.1556</v>
+      </c>
+      <c r="Q178" t="n">
+        <v>0.1556</v>
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="2" t="n">
-        <v>46265</v>
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
@@ -13315,12 +14203,17 @@
         </is>
       </c>
       <c r="P179" t="n">
-        <v>0.955</v>
+        <v>0.0551</v>
+      </c>
+      <c r="Q179" t="n">
+        <v>0.0551</v>
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="2" t="n">
-        <v>46266</v>
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
@@ -13387,12 +14280,17 @@
         </is>
       </c>
       <c r="P180" t="n">
-        <v>0.955</v>
+        <v>0.2298</v>
+      </c>
+      <c r="Q180" t="n">
+        <v>0.2298</v>
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="2" t="n">
-        <v>46266</v>
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
@@ -13459,12 +14357,17 @@
         </is>
       </c>
       <c r="P181" t="n">
-        <v>0.955</v>
+        <v>0.1237</v>
+      </c>
+      <c r="Q181" t="n">
+        <v>0.1237</v>
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="2" t="n">
-        <v>46266</v>
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
@@ -13531,12 +14434,17 @@
         </is>
       </c>
       <c r="P182" t="n">
-        <v>0.955</v>
+        <v>0.1508</v>
+      </c>
+      <c r="Q182" t="n">
+        <v>0.1508</v>
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="2" t="n">
-        <v>46266</v>
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
@@ -13603,12 +14511,17 @@
         </is>
       </c>
       <c r="P183" t="n">
-        <v>0.955</v>
+        <v>0.1508</v>
+      </c>
+      <c r="Q183" t="n">
+        <v>0.1508</v>
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="2" t="n">
-        <v>46266</v>
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
@@ -13675,12 +14588,17 @@
         </is>
       </c>
       <c r="P184" t="n">
-        <v>0.955</v>
+        <v>0.2244</v>
+      </c>
+      <c r="Q184" t="n">
+        <v>0.2244</v>
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="2" t="n">
-        <v>46267</v>
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
@@ -13747,12 +14665,17 @@
         </is>
       </c>
       <c r="P185" t="n">
-        <v>0.955</v>
+        <v>0.1556</v>
+      </c>
+      <c r="Q185" t="n">
+        <v>0.1556</v>
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="2" t="n">
-        <v>46267</v>
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -13819,12 +14742,17 @@
         </is>
       </c>
       <c r="P186" t="n">
-        <v>0.955</v>
+        <v>0.1787</v>
+      </c>
+      <c r="Q186" t="n">
+        <v>0.1787</v>
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="2" t="n">
-        <v>46267</v>
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
@@ -13891,12 +14819,17 @@
         </is>
       </c>
       <c r="P187" t="n">
-        <v>0.955</v>
+        <v>0.1556</v>
+      </c>
+      <c r="Q187" t="n">
+        <v>0.1556</v>
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="2" t="n">
-        <v>46267</v>
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
@@ -13963,12 +14896,17 @@
         </is>
       </c>
       <c r="P188" t="n">
-        <v>0.955</v>
+        <v>0.1462</v>
+      </c>
+      <c r="Q188" t="n">
+        <v>0.1462</v>
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="2" t="n">
-        <v>46267</v>
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
@@ -14035,12 +14973,17 @@
         </is>
       </c>
       <c r="P189" t="n">
-        <v>0.955</v>
+        <v>0.1072</v>
+      </c>
+      <c r="Q189" t="n">
+        <v>0.1072</v>
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="2" t="n">
-        <v>46267</v>
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
@@ -14107,7 +15050,10 @@
         </is>
       </c>
       <c r="P190" t="n">
-        <v>0.955</v>
+        <v>0.1969</v>
+      </c>
+      <c r="Q190" t="n">
+        <v>0.1969</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: adicionar aba comparativa entre Regra Base e Novos Filtros em page 02
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_Odds_Reais_Betfair.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_Odds_Reais_Betfair.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -55,11 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q190"/>
+  <dimension ref="A1:S190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -514,12 +518,20 @@
           <t>P/L</t>
         </is>
       </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Passa_Filtro_Refinado</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Detalhe_Filtro</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
+      <c r="A2" s="2" t="n">
+        <v>46255</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -591,12 +603,18 @@
       <c r="Q2" t="n">
         <v>0.1856</v>
       </c>
+      <c r="R2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Over3.5=2.20 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
+      <c r="A3" s="2" t="n">
+        <v>46255</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -668,12 +686,18 @@
       <c r="Q3" t="n">
         <v>0.1508</v>
       </c>
+      <c r="R3" t="b">
+        <v>0</v>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Over3.5=2.18 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
+      <c r="A4" s="2" t="n">
+        <v>46255</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -745,12 +769,18 @@
       <c r="Q4" t="n">
         <v>0.1856</v>
       </c>
+      <c r="R4" t="b">
+        <v>1</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Over3.5=3.15 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
+      <c r="A5" s="2" t="n">
+        <v>46255</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -822,12 +852,18 @@
       <c r="Q5" t="n">
         <v>0.1379</v>
       </c>
+      <c r="R5" t="b">
+        <v>0</v>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Over3.5=1.52 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
+      <c r="A6" s="2" t="n">
+        <v>46255</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -899,12 +935,18 @@
       <c r="Q6" t="n">
         <v>0.201</v>
       </c>
+      <c r="R6" t="b">
+        <v>1</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Over3.5=2.64 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
+      <c r="A7" s="2" t="n">
+        <v>46255</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -976,12 +1018,18 @@
       <c r="Q7" t="n">
         <v>0.1419</v>
       </c>
+      <c r="R7" t="b">
+        <v>1</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Over3.5=2.58 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
+      <c r="A8" s="2" t="n">
+        <v>46255</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -1053,12 +1101,18 @@
       <c r="Q8" t="n">
         <v>0.2144</v>
       </c>
+      <c r="R8" t="b">
+        <v>1</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Over3.5=3.50 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
+      <c r="A9" s="2" t="n">
+        <v>46255</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1130,12 +1184,18 @@
       <c r="Q9" t="n">
         <v>0.193</v>
       </c>
+      <c r="R9" t="b">
+        <v>0</v>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Over3.5=2.04 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
+      <c r="A10" s="2" t="n">
+        <v>46255</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1207,12 +1267,18 @@
       <c r="Q10" t="n">
         <v>-1</v>
       </c>
+      <c r="R10" t="b">
+        <v>1</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Away=1.61 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
+      <c r="A11" s="2" t="n">
+        <v>46255</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1284,12 +1350,18 @@
       <c r="Q11" t="n">
         <v>0.1508</v>
       </c>
+      <c r="R11" t="b">
+        <v>1</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Away=1.56 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
+      <c r="A12" s="2" t="n">
+        <v>46255</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1361,12 +1433,18 @@
       <c r="Q12" t="n">
         <v>0.1379</v>
       </c>
+      <c r="R12" t="b">
+        <v>0</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Away=1.53 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A13" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1438,12 +1516,18 @@
       <c r="Q13" t="n">
         <v>0.2053</v>
       </c>
+      <c r="R13" t="b">
+        <v>1</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Over3.5=2.54 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A14" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1515,12 +1599,18 @@
       <c r="Q14" t="n">
         <v>0.1556</v>
       </c>
+      <c r="R14" t="b">
+        <v>0</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Over3.5=1.84 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A15" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1592,12 +1682,18 @@
       <c r="Q15" t="n">
         <v>0.201</v>
       </c>
+      <c r="R15" t="b">
+        <v>1</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Over3.5=2.54 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A16" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1669,12 +1765,18 @@
       <c r="Q16" t="n">
         <v>-1</v>
       </c>
+      <c r="R16" t="b">
+        <v>1</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Over3.5=2.78 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A17" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1746,12 +1848,18 @@
       <c r="Q17" t="n">
         <v>0.2053</v>
       </c>
+      <c r="R17" t="b">
+        <v>1</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Over3.5=2.94 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A18" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1823,12 +1931,18 @@
       <c r="Q18" t="n">
         <v>0.1237</v>
       </c>
+      <c r="R18" t="b">
+        <v>0</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Over3.5=2.50 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A19" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1900,12 +2014,18 @@
       <c r="Q19" t="n">
         <v>0.1556</v>
       </c>
+      <c r="R19" t="b">
+        <v>1</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>Over3.5=2.70 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A20" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1977,12 +2097,18 @@
       <c r="Q20" t="n">
         <v>-1</v>
       </c>
+      <c r="R20" t="b">
+        <v>0</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>Over3.5=2.30 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A21" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -2054,12 +2180,18 @@
       <c r="Q21" t="n">
         <v>0.2193</v>
       </c>
+      <c r="R21" t="b">
+        <v>1</v>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>Over3.5=3.10 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A22" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2131,12 +2263,18 @@
       <c r="Q22" t="n">
         <v>0.1419</v>
       </c>
+      <c r="R22" t="b">
+        <v>0</v>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>Over3.5=2.24 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A23" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2208,12 +2346,18 @@
       <c r="Q23" t="n">
         <v>0.1856</v>
       </c>
+      <c r="R23" t="b">
+        <v>1</v>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>Over3.5=2.82 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A24" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2285,12 +2429,18 @@
       <c r="Q24" t="n">
         <v>0.1608</v>
       </c>
+      <c r="R24" t="b">
+        <v>1</v>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Over3.5=3.05 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A25" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2362,12 +2512,18 @@
       <c r="Q25" t="n">
         <v>0.1723</v>
       </c>
+      <c r="R25" t="b">
+        <v>1</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Over3.5=2.56 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A26" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2439,12 +2595,18 @@
       <c r="Q26" t="n">
         <v>0.1856</v>
       </c>
+      <c r="R26" t="b">
+        <v>1</v>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Over3.5=2.80 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A27" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2516,12 +2678,18 @@
       <c r="Q27" t="n">
         <v>0.134</v>
       </c>
+      <c r="R27" t="b">
+        <v>0</v>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>Over3.5=2.26 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A28" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2593,12 +2761,18 @@
       <c r="Q28" t="n">
         <v>0.1723</v>
       </c>
+      <c r="R28" t="b">
+        <v>0</v>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>Over3.5=1.59 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A29" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2670,12 +2844,18 @@
       <c r="Q29" t="n">
         <v>0.1664</v>
       </c>
+      <c r="R29" t="b">
+        <v>1</v>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>Over3.5=2.78 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A30" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2747,12 +2927,18 @@
       <c r="Q30" t="n">
         <v>0.201</v>
       </c>
+      <c r="R30" t="b">
+        <v>0</v>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>Over3.5=2.16 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A31" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2824,12 +3010,18 @@
       <c r="Q31" t="n">
         <v>0.1787</v>
       </c>
+      <c r="R31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Away=1.57 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A32" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2901,12 +3093,18 @@
       <c r="Q32" t="n">
         <v>0.134</v>
       </c>
+      <c r="R32" t="b">
+        <v>0</v>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Away=1.47 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A33" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2978,12 +3176,18 @@
       <c r="Q33" t="n">
         <v>0.2053</v>
       </c>
+      <c r="R33" t="b">
+        <v>1</v>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>Away=1.64 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A34" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -3055,12 +3259,18 @@
       <c r="Q34" t="n">
         <v>0.1149</v>
       </c>
+      <c r="R34" t="b">
+        <v>0</v>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>Away=1.40 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A35" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -3132,12 +3342,18 @@
       <c r="Q35" t="n">
         <v>-1</v>
       </c>
+      <c r="R35" t="b">
+        <v>1</v>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>Away=1.65 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A36" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3209,12 +3425,18 @@
       <c r="Q36" t="n">
         <v>0.127</v>
       </c>
+      <c r="R36" t="b">
+        <v>0</v>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>Away=1.44 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A37" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3286,12 +3508,18 @@
       <c r="Q37" t="n">
         <v>0.1608</v>
       </c>
+      <c r="R37" t="b">
+        <v>1</v>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>Away=1.64 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A38" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3363,12 +3591,18 @@
       <c r="Q38" t="n">
         <v>0.0568</v>
       </c>
+      <c r="R38" t="b">
+        <v>1</v>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>Under &lt;= 1.50</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
+      <c r="A39" s="2" t="n">
+        <v>46256</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3440,12 +3674,18 @@
       <c r="Q39" t="n">
         <v>0.0536</v>
       </c>
+      <c r="R39" t="b">
+        <v>1</v>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Under &lt;= 1.50</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="A40" s="2" t="n">
+        <v>46257</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3517,12 +3757,18 @@
       <c r="Q40" t="n">
         <v>0.1723</v>
       </c>
+      <c r="R40" t="b">
+        <v>0</v>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Over3.5=1.85 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="A41" s="2" t="n">
+        <v>46257</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3594,12 +3840,18 @@
       <c r="Q41" t="n">
         <v>0.193</v>
       </c>
+      <c r="R41" t="b">
+        <v>0</v>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Over3.5=2.36 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="A42" s="2" t="n">
+        <v>46257</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3671,12 +3923,18 @@
       <c r="Q42" t="n">
         <v>0.1664</v>
       </c>
+      <c r="R42" t="b">
+        <v>0</v>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>Over3.5=1.60 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="A43" s="2" t="n">
+        <v>46257</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3748,12 +4006,18 @@
       <c r="Q43" t="n">
         <v>0.1608</v>
       </c>
+      <c r="R43" t="b">
+        <v>0</v>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>Over3.5=1.72 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="A44" s="2" t="n">
+        <v>46257</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3825,12 +4089,18 @@
       <c r="Q44" t="n">
         <v>0.1508</v>
       </c>
+      <c r="R44" t="b">
+        <v>0</v>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>Over3.5=1.90 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="A45" s="2" t="n">
+        <v>46257</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -3902,12 +4172,18 @@
       <c r="Q45" t="n">
         <v>0.1608</v>
       </c>
+      <c r="R45" t="b">
+        <v>0</v>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>Over3.5=1.83 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="A46" s="2" t="n">
+        <v>46257</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -3979,12 +4255,18 @@
       <c r="Q46" t="n">
         <v>0.1462</v>
       </c>
+      <c r="R46" t="b">
+        <v>1</v>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>Over3.5=2.74 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="A47" s="2" t="n">
+        <v>46257</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -4056,12 +4338,18 @@
       <c r="Q47" t="n">
         <v>0.1237</v>
       </c>
+      <c r="R47" t="b">
+        <v>0</v>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>Over3.5=2.04 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="A48" s="2" t="n">
+        <v>46257</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -4133,12 +4421,18 @@
       <c r="Q48" t="n">
         <v>0.1379</v>
       </c>
+      <c r="R48" t="b">
+        <v>1</v>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>Over3.5=2.88 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="A49" s="2" t="n">
+        <v>46257</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -4210,12 +4504,18 @@
       <c r="Q49" t="n">
         <v>0.1664</v>
       </c>
+      <c r="R49" t="b">
+        <v>0</v>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>Over3.5=1.64 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="A50" s="2" t="n">
+        <v>46257</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -4287,12 +4587,18 @@
       <c r="Q50" t="n">
         <v>0.1723</v>
       </c>
+      <c r="R50" t="b">
+        <v>1</v>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>Over3.5=2.82 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="A51" s="2" t="n">
+        <v>46257</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -4364,12 +4670,18 @@
       <c r="Q51" t="n">
         <v>0.1856</v>
       </c>
+      <c r="R51" t="b">
+        <v>0</v>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>Over3.5=2.34 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="A52" s="2" t="n">
+        <v>46257</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -4441,12 +4753,18 @@
       <c r="Q52" t="n">
         <v>0.1664</v>
       </c>
+      <c r="R52" t="b">
+        <v>1</v>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Over3.5=2.88 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="A53" s="2" t="n">
+        <v>46257</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -4518,12 +4836,18 @@
       <c r="Q53" t="n">
         <v>-1</v>
       </c>
+      <c r="R53" t="b">
+        <v>1</v>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Away=1.61 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="A54" s="2" t="n">
+        <v>46257</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -4595,12 +4919,18 @@
       <c r="Q54" t="n">
         <v>0.2053</v>
       </c>
+      <c r="R54" t="b">
+        <v>1</v>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>Away=1.59 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="A55" s="2" t="n">
+        <v>46257</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -4672,12 +5002,18 @@
       <c r="Q55" t="n">
         <v>0.1556</v>
       </c>
+      <c r="R55" t="b">
+        <v>1</v>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>Away=1.61 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="A56" s="2" t="n">
+        <v>46257</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -4749,12 +5085,18 @@
       <c r="Q56" t="n">
         <v>0.1304</v>
       </c>
+      <c r="R56" t="b">
+        <v>0</v>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>Away=1.48 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="A57" s="2" t="n">
+        <v>46257</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -4826,12 +5168,18 @@
       <c r="Q57" t="n">
         <v>0.127</v>
       </c>
+      <c r="R57" t="b">
+        <v>0</v>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>Away=1.50 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="A58" s="2" t="n">
+        <v>46257</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -4903,12 +5251,18 @@
       <c r="Q58" t="n">
         <v>0.1608</v>
       </c>
+      <c r="R58" t="b">
+        <v>0</v>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>Away=1.50 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="A59" s="2" t="n">
+        <v>46257</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -4980,12 +5334,18 @@
       <c r="Q59" t="n">
         <v>0.1379</v>
       </c>
+      <c r="R59" t="b">
+        <v>0</v>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>Away=1.44 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="A60" s="2" t="n">
+        <v>46257</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -5057,12 +5417,18 @@
       <c r="Q60" t="n">
         <v>0.1122</v>
       </c>
+      <c r="R60" t="b">
+        <v>0</v>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>Away=1.37 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="A61" s="2" t="n">
+        <v>46257</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -5134,12 +5500,18 @@
       <c r="Q61" t="n">
         <v>0.1787</v>
       </c>
+      <c r="R61" t="b">
+        <v>1</v>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>Away=1.61 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
+      <c r="A62" s="2" t="n">
+        <v>46257</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -5211,12 +5583,18 @@
       <c r="Q62" t="n">
         <v>0.0568</v>
       </c>
+      <c r="R62" t="b">
+        <v>1</v>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>Under &lt;= 1.50</t>
+        </is>
+      </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
+      <c r="A63" s="2" t="n">
+        <v>46258</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -5288,12 +5666,18 @@
       <c r="Q63" t="n">
         <v>0.2193</v>
       </c>
+      <c r="R63" t="b">
+        <v>1</v>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>Over3.5=2.96 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
+      <c r="A64" s="2" t="n">
+        <v>46258</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -5365,12 +5749,18 @@
       <c r="Q64" t="n">
         <v>0.2193</v>
       </c>
+      <c r="R64" t="b">
+        <v>1</v>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>Over3.5=3.05 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
+      <c r="A65" s="2" t="n">
+        <v>46258</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -5442,12 +5832,18 @@
       <c r="Q65" t="n">
         <v>0.1608</v>
       </c>
+      <c r="R65" t="b">
+        <v>0</v>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>Away=1.51 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
+      <c r="A66" s="2" t="n">
+        <v>46258</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -5519,12 +5915,18 @@
       <c r="Q66" t="n">
         <v>0.1664</v>
       </c>
+      <c r="R66" t="b">
+        <v>0</v>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>Away=1.52 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
+      <c r="A67" s="2" t="n">
+        <v>46259</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -5596,12 +5998,18 @@
       <c r="Q67" t="n">
         <v>0.2193</v>
       </c>
+      <c r="R67" t="b">
+        <v>1</v>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>Over3.5=3.85 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
+      <c r="A68" s="2" t="n">
+        <v>46259</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -5673,12 +6081,18 @@
       <c r="Q68" t="n">
         <v>0.1462</v>
       </c>
+      <c r="R68" t="b">
+        <v>0</v>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>Over3.5=1.83 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
+      <c r="A69" s="2" t="n">
+        <v>46259</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -5750,12 +6164,18 @@
       <c r="Q69" t="n">
         <v>0.1206</v>
       </c>
+      <c r="R69" t="b">
+        <v>0</v>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>Over3.5=1.60 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
+      <c r="A70" s="2" t="n">
+        <v>46259</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -5827,12 +6247,18 @@
       <c r="Q70" t="n">
         <v>0.1856</v>
       </c>
+      <c r="R70" t="b">
+        <v>1</v>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>Away=1.62 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
+      <c r="A71" s="2" t="n">
+        <v>46259</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -5904,12 +6330,18 @@
       <c r="Q71" t="n">
         <v>0.1723</v>
       </c>
+      <c r="R71" t="b">
+        <v>1</v>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>Away=1.61 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
+      <c r="A72" s="2" t="n">
+        <v>46259</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -5981,12 +6413,18 @@
       <c r="Q72" t="n">
         <v>0.0551</v>
       </c>
+      <c r="R72" t="b">
+        <v>1</v>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>Under &lt;= 1.50</t>
+        </is>
+      </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
+      <c r="A73" s="2" t="n">
+        <v>46259</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -6052,12 +6490,18 @@
       <c r="Q73" t="n">
         <v>0</v>
       </c>
+      <c r="R73" t="b">
+        <v>1</v>
+      </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>Under &lt;= 1.50</t>
+        </is>
+      </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
+      <c r="A74" s="2" t="n">
+        <v>46260</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -6129,12 +6573,18 @@
       <c r="Q74" t="n">
         <v>0.134</v>
       </c>
+      <c r="R74" t="b">
+        <v>0</v>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>Over3.5=1.87 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
+      <c r="A75" s="2" t="n">
+        <v>46260</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -6206,12 +6656,18 @@
       <c r="Q75" t="n">
         <v>0.1787</v>
       </c>
+      <c r="R75" t="b">
+        <v>1</v>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>Over3.5=3.20 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
+      <c r="A76" s="2" t="n">
+        <v>46260</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
@@ -6283,12 +6739,18 @@
       <c r="Q76" t="n">
         <v>0.193</v>
       </c>
+      <c r="R76" t="b">
+        <v>0</v>
+      </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>Over3.5=2.30 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
+      <c r="A77" s="2" t="n">
+        <v>46260</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
@@ -6360,12 +6822,18 @@
       <c r="Q77" t="n">
         <v>0.1608</v>
       </c>
+      <c r="R77" t="b">
+        <v>0</v>
+      </c>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>Over3.5=2.20 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
+      <c r="A78" s="2" t="n">
+        <v>46260</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
@@ -6437,12 +6905,18 @@
       <c r="Q78" t="n">
         <v>0.1664</v>
       </c>
+      <c r="R78" t="b">
+        <v>0</v>
+      </c>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>Over3.5=2.06 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
+      <c r="A79" s="2" t="n">
+        <v>46260</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -6514,12 +6988,18 @@
       <c r="Q79" t="n">
         <v>0.1969</v>
       </c>
+      <c r="R79" t="b">
+        <v>0</v>
+      </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>Over3.5=2.48 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
+      <c r="A80" s="2" t="n">
+        <v>46260</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -6585,12 +7065,18 @@
       <c r="Q80" t="n">
         <v>0</v>
       </c>
+      <c r="R80" t="b">
+        <v>0</v>
+      </c>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>Over3.5=1.05 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
+      <c r="A81" s="2" t="n">
+        <v>46260</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -6662,12 +7148,18 @@
       <c r="Q81" t="n">
         <v>-1</v>
       </c>
+      <c r="R81" t="b">
+        <v>0</v>
+      </c>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>Over3.5=1.67 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
+      <c r="A82" s="2" t="n">
+        <v>46260</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -6739,12 +7231,18 @@
       <c r="Q82" t="n">
         <v>-1</v>
       </c>
+      <c r="R82" t="b">
+        <v>1</v>
+      </c>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>Over3.5=4.30 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
+      <c r="A83" s="2" t="n">
+        <v>46260</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
@@ -6816,12 +7314,18 @@
       <c r="Q83" t="n">
         <v>0.1556</v>
       </c>
+      <c r="R83" t="b">
+        <v>1</v>
+      </c>
+      <c r="S83" t="inlineStr">
+        <is>
+          <t>Away=1.55 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
+      <c r="A84" s="2" t="n">
+        <v>46260</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -6893,12 +7397,18 @@
       <c r="Q84" t="n">
         <v>0.0522</v>
       </c>
+      <c r="R84" t="b">
+        <v>1</v>
+      </c>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>Under &lt;= 1.50</t>
+        </is>
+      </c>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
+      <c r="A85" s="2" t="n">
+        <v>46261</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
@@ -6970,12 +7480,18 @@
       <c r="Q85" t="n">
         <v>0.1177</v>
       </c>
+      <c r="R85" t="b">
+        <v>0</v>
+      </c>
+      <c r="S85" t="inlineStr">
+        <is>
+          <t>Over3.5=2.18 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
+      <c r="A86" s="2" t="n">
+        <v>46261</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
@@ -7047,12 +7563,18 @@
       <c r="Q86" t="n">
         <v>0.1787</v>
       </c>
+      <c r="R86" t="b">
+        <v>0</v>
+      </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>Over3.5=2.46 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
+      <c r="A87" s="2" t="n">
+        <v>46261</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
@@ -7124,12 +7646,18 @@
       <c r="Q87" t="n">
         <v>0.1856</v>
       </c>
+      <c r="R87" t="b">
+        <v>1</v>
+      </c>
+      <c r="S87" t="inlineStr">
+        <is>
+          <t>Over3.5=2.72 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
+      <c r="A88" s="2" t="n">
+        <v>46261</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -7201,12 +7729,18 @@
       <c r="Q88" t="n">
         <v>0.2193</v>
       </c>
+      <c r="R88" t="b">
+        <v>1</v>
+      </c>
+      <c r="S88" t="inlineStr">
+        <is>
+          <t>Over3.5=3.05 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
+      <c r="A89" s="2" t="n">
+        <v>46261</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
@@ -7278,12 +7812,18 @@
       <c r="Q89" t="n">
         <v>0.1462</v>
       </c>
+      <c r="R89" t="b">
+        <v>0</v>
+      </c>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t>Over3.5=2.20 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
+      <c r="A90" s="2" t="n">
+        <v>46261</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
@@ -7355,12 +7895,18 @@
       <c r="Q90" t="n">
         <v>0.1723</v>
       </c>
+      <c r="R90" t="b">
+        <v>0</v>
+      </c>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>Over3.5=1.84 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
+      <c r="A91" s="2" t="n">
+        <v>46261</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
@@ -7432,12 +7978,18 @@
       <c r="Q91" t="n">
         <v>0.1072</v>
       </c>
+      <c r="R91" t="b">
+        <v>0</v>
+      </c>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t>Over3.5=1.87 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
+      <c r="A92" s="2" t="n">
+        <v>46261</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
@@ -7509,12 +8061,18 @@
       <c r="Q92" t="n">
         <v>0.1462</v>
       </c>
+      <c r="R92" t="b">
+        <v>0</v>
+      </c>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t>Over3.5=2.30 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
+      <c r="A93" s="2" t="n">
+        <v>46261</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
@@ -7586,12 +8144,18 @@
       <c r="Q93" t="n">
         <v>0.2098</v>
       </c>
+      <c r="R93" t="b">
+        <v>1</v>
+      </c>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>Over3.5=2.90 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
+      <c r="A94" s="2" t="n">
+        <v>46261</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
@@ -7663,12 +8227,18 @@
       <c r="Q94" t="n">
         <v>-1</v>
       </c>
+      <c r="R94" t="b">
+        <v>0</v>
+      </c>
+      <c r="S94" t="inlineStr">
+        <is>
+          <t>Over3.5=2.08 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
+      <c r="A95" s="2" t="n">
+        <v>46261</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
@@ -7740,12 +8310,18 @@
       <c r="Q95" t="n">
         <v>0.1419</v>
       </c>
+      <c r="R95" t="b">
+        <v>0</v>
+      </c>
+      <c r="S95" t="inlineStr">
+        <is>
+          <t>Over3.5=2.08 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
+      <c r="A96" s="2" t="n">
+        <v>46261</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
@@ -7817,12 +8393,18 @@
       <c r="Q96" t="n">
         <v>0.1419</v>
       </c>
+      <c r="R96" t="b">
+        <v>0</v>
+      </c>
+      <c r="S96" t="inlineStr">
+        <is>
+          <t>Over3.5=2.02 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
+      <c r="A97" s="2" t="n">
+        <v>46261</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
@@ -7894,12 +8476,18 @@
       <c r="Q97" t="n">
         <v>-1</v>
       </c>
+      <c r="R97" t="b">
+        <v>0</v>
+      </c>
+      <c r="S97" t="inlineStr">
+        <is>
+          <t>Away=1.40 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
+      <c r="A98" s="2" t="n">
+        <v>46261</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -7971,12 +8559,18 @@
       <c r="Q98" t="n">
         <v>0.1462</v>
       </c>
+      <c r="R98" t="b">
+        <v>0</v>
+      </c>
+      <c r="S98" t="inlineStr">
+        <is>
+          <t>Away=1.51 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
+      <c r="A99" s="2" t="n">
+        <v>46261</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
@@ -8048,12 +8642,18 @@
       <c r="Q99" t="n">
         <v>0.1379</v>
       </c>
+      <c r="R99" t="b">
+        <v>0</v>
+      </c>
+      <c r="S99" t="inlineStr">
+        <is>
+          <t>Away=1.44 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
+      <c r="A100" s="2" t="n">
+        <v>46261</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
@@ -8125,12 +8725,18 @@
       <c r="Q100" t="n">
         <v>0.1072</v>
       </c>
+      <c r="R100" t="b">
+        <v>0</v>
+      </c>
+      <c r="S100" t="inlineStr">
+        <is>
+          <t>Away=1.42 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
+      <c r="A101" s="2" t="n">
+        <v>46261</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
@@ -8202,12 +8808,18 @@
       <c r="Q101" t="n">
         <v>0.0568</v>
       </c>
+      <c r="R101" t="b">
+        <v>1</v>
+      </c>
+      <c r="S101" t="inlineStr">
+        <is>
+          <t>Under &lt;= 1.50</t>
+        </is>
+      </c>
     </row>
     <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
+      <c r="A102" s="2" t="n">
+        <v>46262</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
@@ -8279,12 +8891,18 @@
       <c r="Q102" t="n">
         <v>0.1723</v>
       </c>
+      <c r="R102" t="b">
+        <v>0</v>
+      </c>
+      <c r="S102" t="inlineStr">
+        <is>
+          <t>Over3.5=2.52 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
+      <c r="A103" s="2" t="n">
+        <v>46262</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -8356,12 +8974,18 @@
       <c r="Q103" t="n">
         <v>0.1664</v>
       </c>
+      <c r="R103" t="b">
+        <v>0</v>
+      </c>
+      <c r="S103" t="inlineStr">
+        <is>
+          <t>Over3.5=1.98 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
+      <c r="A104" s="2" t="n">
+        <v>46262</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -8433,12 +9057,18 @@
       <c r="Q104" t="n">
         <v>0.1304</v>
       </c>
+      <c r="R104" t="b">
+        <v>0</v>
+      </c>
+      <c r="S104" t="inlineStr">
+        <is>
+          <t>Over3.5=1.49 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
+      <c r="A105" s="2" t="n">
+        <v>46262</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
@@ -8510,12 +9140,18 @@
       <c r="Q105" t="n">
         <v>0.1723</v>
       </c>
+      <c r="R105" t="b">
+        <v>0</v>
+      </c>
+      <c r="S105" t="inlineStr">
+        <is>
+          <t>Over3.5=2.22 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
+      <c r="A106" s="2" t="n">
+        <v>46262</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
@@ -8587,12 +9223,18 @@
       <c r="Q106" t="n">
         <v>0.1379</v>
       </c>
+      <c r="R106" t="b">
+        <v>0</v>
+      </c>
+      <c r="S106" t="inlineStr">
+        <is>
+          <t>Over3.5=1.99 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
+      <c r="A107" s="2" t="n">
+        <v>46262</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
@@ -8664,12 +9306,18 @@
       <c r="Q107" t="n">
         <v>0.1664</v>
       </c>
+      <c r="R107" t="b">
+        <v>0</v>
+      </c>
+      <c r="S107" t="inlineStr">
+        <is>
+          <t>Over3.5=2.40 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
+      <c r="A108" s="2" t="n">
+        <v>46262</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
@@ -8741,12 +9389,18 @@
       <c r="Q108" t="n">
         <v>0.2053</v>
       </c>
+      <c r="R108" t="b">
+        <v>0</v>
+      </c>
+      <c r="S108" t="inlineStr">
+        <is>
+          <t>Over3.5=2.44 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
+      <c r="A109" s="2" t="n">
+        <v>46262</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
@@ -8818,12 +9472,18 @@
       <c r="Q109" t="n">
         <v>0.127</v>
       </c>
+      <c r="R109" t="b">
+        <v>0</v>
+      </c>
+      <c r="S109" t="inlineStr">
+        <is>
+          <t>Over3.5=2.04 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
+      <c r="A110" s="2" t="n">
+        <v>46262</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
@@ -8895,12 +9555,18 @@
       <c r="Q110" t="n">
         <v>0.1608</v>
       </c>
+      <c r="R110" t="b">
+        <v>0</v>
+      </c>
+      <c r="S110" t="inlineStr">
+        <is>
+          <t>Over3.5=2.44 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
+      <c r="A111" s="2" t="n">
+        <v>46262</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
@@ -8972,12 +9638,18 @@
       <c r="Q111" t="n">
         <v>0.1664</v>
       </c>
+      <c r="R111" t="b">
+        <v>0</v>
+      </c>
+      <c r="S111" t="inlineStr">
+        <is>
+          <t>Over3.5=1.65 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
+      <c r="A112" s="2" t="n">
+        <v>46262</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
@@ -9049,12 +9721,18 @@
       <c r="Q112" t="n">
         <v>0.201</v>
       </c>
+      <c r="R112" t="b">
+        <v>1</v>
+      </c>
+      <c r="S112" t="inlineStr">
+        <is>
+          <t>Over3.5=2.62 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
+      <c r="A113" s="2" t="n">
+        <v>46262</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
@@ -9126,12 +9804,18 @@
       <c r="Q113" t="n">
         <v>0.134</v>
       </c>
+      <c r="R113" t="b">
+        <v>0</v>
+      </c>
+      <c r="S113" t="inlineStr">
+        <is>
+          <t>Away=1.43 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
+      <c r="A114" s="2" t="n">
+        <v>46262</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
@@ -9203,12 +9887,18 @@
       <c r="Q114" t="n">
         <v>0.1664</v>
       </c>
+      <c r="R114" t="b">
+        <v>1</v>
+      </c>
+      <c r="S114" t="inlineStr">
+        <is>
+          <t>Away=1.59 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
+      <c r="A115" s="2" t="n">
+        <v>46262</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
@@ -9280,12 +9970,18 @@
       <c r="Q115" t="n">
         <v>0.0508</v>
       </c>
+      <c r="R115" t="b">
+        <v>1</v>
+      </c>
+      <c r="S115" t="inlineStr">
+        <is>
+          <t>Under &lt;= 1.50</t>
+        </is>
+      </c>
     </row>
     <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
+      <c r="A116" s="2" t="n">
+        <v>46263</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
@@ -9357,12 +10053,18 @@
       <c r="Q116" t="n">
         <v>0.1608</v>
       </c>
+      <c r="R116" t="b">
+        <v>1</v>
+      </c>
+      <c r="S116" t="inlineStr">
+        <is>
+          <t>Over3.5=2.70 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
+      <c r="A117" s="2" t="n">
+        <v>46263</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
@@ -9434,12 +10136,18 @@
       <c r="Q117" t="n">
         <v>0.1856</v>
       </c>
+      <c r="R117" t="b">
+        <v>0</v>
+      </c>
+      <c r="S117" t="inlineStr">
+        <is>
+          <t>Over3.5=2.18 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
+      <c r="A118" s="2" t="n">
+        <v>46263</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
@@ -9511,12 +10219,18 @@
       <c r="Q118" t="n">
         <v>0.1097</v>
       </c>
+      <c r="R118" t="b">
+        <v>0</v>
+      </c>
+      <c r="S118" t="inlineStr">
+        <is>
+          <t>Over3.5=1.77 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
+      <c r="A119" s="2" t="n">
+        <v>46263</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
@@ -9588,12 +10302,18 @@
       <c r="Q119" t="n">
         <v>-1</v>
       </c>
+      <c r="R119" t="b">
+        <v>1</v>
+      </c>
+      <c r="S119" t="inlineStr">
+        <is>
+          <t>Over3.5=2.88 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
+      <c r="A120" s="2" t="n">
+        <v>46263</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
@@ -9665,12 +10385,18 @@
       <c r="Q120" t="n">
         <v>0.1608</v>
       </c>
+      <c r="R120" t="b">
+        <v>0</v>
+      </c>
+      <c r="S120" t="inlineStr">
+        <is>
+          <t>Over3.5=2.30 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
+      <c r="A121" s="2" t="n">
+        <v>46263</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
@@ -9742,12 +10468,18 @@
       <c r="Q121" t="n">
         <v>0.193</v>
       </c>
+      <c r="R121" t="b">
+        <v>0</v>
+      </c>
+      <c r="S121" t="inlineStr">
+        <is>
+          <t>Over3.5=1.98 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
+      <c r="A122" s="2" t="n">
+        <v>46263</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
@@ -9819,12 +10551,18 @@
       <c r="Q122" t="n">
         <v>0.1787</v>
       </c>
+      <c r="R122" t="b">
+        <v>1</v>
+      </c>
+      <c r="S122" t="inlineStr">
+        <is>
+          <t>Over3.5=2.88 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
+      <c r="A123" s="2" t="n">
+        <v>46263</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
@@ -9896,12 +10634,18 @@
       <c r="Q123" t="n">
         <v>0.1787</v>
       </c>
+      <c r="R123" t="b">
+        <v>0</v>
+      </c>
+      <c r="S123" t="inlineStr">
+        <is>
+          <t>Over3.5=2.36 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
+      <c r="A124" s="2" t="n">
+        <v>46263</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -9973,12 +10717,18 @@
       <c r="Q124" t="n">
         <v>0.1664</v>
       </c>
+      <c r="R124" t="b">
+        <v>1</v>
+      </c>
+      <c r="S124" t="inlineStr">
+        <is>
+          <t>Over3.5=3.05 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
+      <c r="A125" s="2" t="n">
+        <v>46263</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -10050,12 +10800,18 @@
       <c r="Q125" t="n">
         <v>0.1664</v>
       </c>
+      <c r="R125" t="b">
+        <v>1</v>
+      </c>
+      <c r="S125" t="inlineStr">
+        <is>
+          <t>Over3.5=2.66 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
+      <c r="A126" s="2" t="n">
+        <v>46263</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -10127,12 +10883,18 @@
       <c r="Q126" t="n">
         <v>0.1664</v>
       </c>
+      <c r="R126" t="b">
+        <v>1</v>
+      </c>
+      <c r="S126" t="inlineStr">
+        <is>
+          <t>Over3.5=3.10 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
+      <c r="A127" s="2" t="n">
+        <v>46263</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -10204,12 +10966,18 @@
       <c r="Q127" t="n">
         <v>0.2144</v>
       </c>
+      <c r="R127" t="b">
+        <v>1</v>
+      </c>
+      <c r="S127" t="inlineStr">
+        <is>
+          <t>Over3.5=3.45 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
+      <c r="A128" s="2" t="n">
+        <v>46263</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
@@ -10281,12 +11049,18 @@
       <c r="Q128" t="n">
         <v>0.1856</v>
       </c>
+      <c r="R128" t="b">
+        <v>1</v>
+      </c>
+      <c r="S128" t="inlineStr">
+        <is>
+          <t>Away=1.62 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
+      <c r="A129" s="2" t="n">
+        <v>46263</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -10358,12 +11132,18 @@
       <c r="Q129" t="n">
         <v>0.201</v>
       </c>
+      <c r="R129" t="b">
+        <v>1</v>
+      </c>
+      <c r="S129" t="inlineStr">
+        <is>
+          <t>Away=1.63 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
+      <c r="A130" s="2" t="n">
+        <v>46263</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
@@ -10435,12 +11215,18 @@
       <c r="Q130" t="n">
         <v>0.1206</v>
       </c>
+      <c r="R130" t="b">
+        <v>0</v>
+      </c>
+      <c r="S130" t="inlineStr">
+        <is>
+          <t>Away=1.44 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
+      <c r="A131" s="2" t="n">
+        <v>46263</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
@@ -10512,12 +11298,18 @@
       <c r="Q131" t="n">
         <v>0.1379</v>
       </c>
+      <c r="R131" t="b">
+        <v>0</v>
+      </c>
+      <c r="S131" t="inlineStr">
+        <is>
+          <t>Away=1.45 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
+      <c r="A132" s="2" t="n">
+        <v>46263</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
@@ -10589,12 +11381,18 @@
       <c r="Q132" t="n">
         <v>0.1304</v>
       </c>
+      <c r="R132" t="b">
+        <v>0</v>
+      </c>
+      <c r="S132" t="inlineStr">
+        <is>
+          <t>Away=1.48 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="133">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
+      <c r="A133" s="2" t="n">
+        <v>46263</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
@@ -10666,12 +11464,18 @@
       <c r="Q133" t="n">
         <v>0.1462</v>
       </c>
+      <c r="R133" t="b">
+        <v>0</v>
+      </c>
+      <c r="S133" t="inlineStr">
+        <is>
+          <t>Away=1.46 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
+      <c r="A134" s="2" t="n">
+        <v>46263</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
@@ -10743,12 +11547,18 @@
       <c r="Q134" t="n">
         <v>0.0568</v>
       </c>
+      <c r="R134" t="b">
+        <v>1</v>
+      </c>
+      <c r="S134" t="inlineStr">
+        <is>
+          <t>Under &lt;= 1.50</t>
+        </is>
+      </c>
     </row>
     <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
+      <c r="A135" s="2" t="n">
+        <v>46263</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
@@ -10820,12 +11630,18 @@
       <c r="Q135" t="n">
         <v>0.1016</v>
       </c>
+      <c r="R135" t="b">
+        <v>1</v>
+      </c>
+      <c r="S135" t="inlineStr">
+        <is>
+          <t>Under &lt;= 1.50</t>
+        </is>
+      </c>
     </row>
     <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
+      <c r="A136" s="2" t="n">
+        <v>46263</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -10897,12 +11713,18 @@
       <c r="Q136" t="n">
         <v>0.0551</v>
       </c>
+      <c r="R136" t="b">
+        <v>1</v>
+      </c>
+      <c r="S136" t="inlineStr">
+        <is>
+          <t>Under &lt;= 1.50</t>
+        </is>
+      </c>
     </row>
     <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A137" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
@@ -10974,12 +11796,18 @@
       <c r="Q137" t="n">
         <v>0.193</v>
       </c>
+      <c r="R137" t="b">
+        <v>0</v>
+      </c>
+      <c r="S137" t="inlineStr">
+        <is>
+          <t>Over3.5=2.44 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A138" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
@@ -11051,12 +11879,18 @@
       <c r="Q138" t="n">
         <v>-1</v>
       </c>
+      <c r="R138" t="b">
+        <v>0</v>
+      </c>
+      <c r="S138" t="inlineStr">
+        <is>
+          <t>Over3.5=1.73 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A139" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
@@ -11128,12 +11962,18 @@
       <c r="Q139" t="n">
         <v>0.1664</v>
       </c>
+      <c r="R139" t="b">
+        <v>0</v>
+      </c>
+      <c r="S139" t="inlineStr">
+        <is>
+          <t>Over3.5=1.79 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A140" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
@@ -11205,12 +12045,18 @@
       <c r="Q140" t="n">
         <v>0.193</v>
       </c>
+      <c r="R140" t="b">
+        <v>1</v>
+      </c>
+      <c r="S140" t="inlineStr">
+        <is>
+          <t>Over3.5=2.74 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A141" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
@@ -11282,12 +12128,18 @@
       <c r="Q141" t="n">
         <v>0.1664</v>
       </c>
+      <c r="R141" t="b">
+        <v>0</v>
+      </c>
+      <c r="S141" t="inlineStr">
+        <is>
+          <t>Over3.5=1.67 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A142" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
@@ -11359,12 +12211,18 @@
       <c r="Q142" t="n">
         <v>0.1608</v>
       </c>
+      <c r="R142" t="b">
+        <v>0</v>
+      </c>
+      <c r="S142" t="inlineStr">
+        <is>
+          <t>Over3.5=1.95 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A143" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
@@ -11436,12 +12294,18 @@
       <c r="Q143" t="n">
         <v>0.201</v>
       </c>
+      <c r="R143" t="b">
+        <v>0</v>
+      </c>
+      <c r="S143" t="inlineStr">
+        <is>
+          <t>Over3.5=2.18 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A144" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
@@ -11513,12 +12377,18 @@
       <c r="Q144" t="n">
         <v>0.1969</v>
       </c>
+      <c r="R144" t="b">
+        <v>0</v>
+      </c>
+      <c r="S144" t="inlineStr">
+        <is>
+          <t>Over3.5=2.28 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A145" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
@@ -11590,12 +12460,18 @@
       <c r="Q145" t="n">
         <v>0.1723</v>
       </c>
+      <c r="R145" t="b">
+        <v>1</v>
+      </c>
+      <c r="S145" t="inlineStr">
+        <is>
+          <t>Over3.5=2.54 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A146" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
@@ -11667,12 +12543,18 @@
       <c r="Q146" t="n">
         <v>0.1723</v>
       </c>
+      <c r="R146" t="b">
+        <v>0</v>
+      </c>
+      <c r="S146" t="inlineStr">
+        <is>
+          <t>Over3.5=1.93 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A147" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
@@ -11744,12 +12626,18 @@
       <c r="Q147" t="n">
         <v>-1</v>
       </c>
+      <c r="R147" t="b">
+        <v>1</v>
+      </c>
+      <c r="S147" t="inlineStr">
+        <is>
+          <t>Over3.5=3.05 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A148" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
@@ -11821,12 +12709,18 @@
       <c r="Q148" t="n">
         <v>0.1097</v>
       </c>
+      <c r="R148" t="b">
+        <v>0</v>
+      </c>
+      <c r="S148" t="inlineStr">
+        <is>
+          <t>Over3.5=1.76 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A149" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
@@ -11898,12 +12792,18 @@
       <c r="Q149" t="n">
         <v>-1</v>
       </c>
+      <c r="R149" t="b">
+        <v>1</v>
+      </c>
+      <c r="S149" t="inlineStr">
+        <is>
+          <t>Over3.5=3.30 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A150" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
@@ -11975,12 +12875,18 @@
       <c r="Q150" t="n">
         <v>0.201</v>
       </c>
+      <c r="R150" t="b">
+        <v>1</v>
+      </c>
+      <c r="S150" t="inlineStr">
+        <is>
+          <t>Over3.5=2.68 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A151" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
@@ -12052,12 +12958,18 @@
       <c r="Q151" t="n">
         <v>0.1177</v>
       </c>
+      <c r="R151" t="b">
+        <v>0</v>
+      </c>
+      <c r="S151" t="inlineStr">
+        <is>
+          <t>Over3.5=2.28 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A152" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
@@ -12129,12 +13041,18 @@
       <c r="Q152" t="n">
         <v>-1</v>
       </c>
+      <c r="R152" t="b">
+        <v>1</v>
+      </c>
+      <c r="S152" t="inlineStr">
+        <is>
+          <t>Over3.5=3.30 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A153" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
@@ -12206,12 +13124,18 @@
       <c r="Q153" t="n">
         <v>0.1723</v>
       </c>
+      <c r="R153" t="b">
+        <v>0</v>
+      </c>
+      <c r="S153" t="inlineStr">
+        <is>
+          <t>Over3.5=2.20 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A154" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
@@ -12283,12 +13207,18 @@
       <c r="Q154" t="n">
         <v>0.201</v>
       </c>
+      <c r="R154" t="b">
+        <v>1</v>
+      </c>
+      <c r="S154" t="inlineStr">
+        <is>
+          <t>Away=1.60 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A155" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
@@ -12360,12 +13290,18 @@
       <c r="Q155" t="n">
         <v>0.1379</v>
       </c>
+      <c r="R155" t="b">
+        <v>0</v>
+      </c>
+      <c r="S155" t="inlineStr">
+        <is>
+          <t>Away=1.51 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A156" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
@@ -12437,12 +13373,18 @@
       <c r="Q156" t="n">
         <v>0.1508</v>
       </c>
+      <c r="R156" t="b">
+        <v>1</v>
+      </c>
+      <c r="S156" t="inlineStr">
+        <is>
+          <t>Away=1.56 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A157" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
@@ -12514,12 +13456,18 @@
       <c r="Q157" t="n">
         <v>0.1664</v>
       </c>
+      <c r="R157" t="b">
+        <v>0</v>
+      </c>
+      <c r="S157" t="inlineStr">
+        <is>
+          <t>Away=1.52 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A158" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
@@ -12591,12 +13539,18 @@
       <c r="Q158" t="n">
         <v>0.1664</v>
       </c>
+      <c r="R158" t="b">
+        <v>0</v>
+      </c>
+      <c r="S158" t="inlineStr">
+        <is>
+          <t>Away=1.53 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A159" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
@@ -12668,12 +13622,18 @@
       <c r="Q159" t="n">
         <v>0.1787</v>
       </c>
+      <c r="R159" t="b">
+        <v>1</v>
+      </c>
+      <c r="S159" t="inlineStr">
+        <is>
+          <t>Away=1.55 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A160" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
@@ -12745,12 +13705,18 @@
       <c r="Q160" t="n">
         <v>0.2053</v>
       </c>
+      <c r="R160" t="b">
+        <v>1</v>
+      </c>
+      <c r="S160" t="inlineStr">
+        <is>
+          <t>Away=1.58 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A161" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
@@ -12822,12 +13788,18 @@
       <c r="Q161" t="n">
         <v>0.2298</v>
       </c>
+      <c r="R161" t="b">
+        <v>1</v>
+      </c>
+      <c r="S161" t="inlineStr">
+        <is>
+          <t>Away=1.58 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="162">
-      <c r="A162" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A162" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
@@ -12899,12 +13871,18 @@
       <c r="Q162" t="n">
         <v>0.1664</v>
       </c>
+      <c r="R162" t="b">
+        <v>1</v>
+      </c>
+      <c r="S162" t="inlineStr">
+        <is>
+          <t>Away=1.61 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="163">
-      <c r="A163" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A163" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
@@ -12976,12 +13954,18 @@
       <c r="Q163" t="n">
         <v>0.1608</v>
       </c>
+      <c r="R163" t="b">
+        <v>1</v>
+      </c>
+      <c r="S163" t="inlineStr">
+        <is>
+          <t>Away=1.60 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A164" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B164" t="inlineStr">
         <is>
@@ -13053,12 +14037,18 @@
       <c r="Q164" t="n">
         <v>0.1856</v>
       </c>
+      <c r="R164" t="b">
+        <v>1</v>
+      </c>
+      <c r="S164" t="inlineStr">
+        <is>
+          <t>Away=1.65 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="165">
-      <c r="A165" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A165" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
@@ -13130,12 +14120,18 @@
       <c r="Q165" t="n">
         <v>0.1462</v>
       </c>
+      <c r="R165" t="b">
+        <v>1</v>
+      </c>
+      <c r="S165" t="inlineStr">
+        <is>
+          <t>Away=1.62 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="166">
-      <c r="A166" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A166" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B166" t="inlineStr">
         <is>
@@ -13207,12 +14203,18 @@
       <c r="Q166" t="n">
         <v>0.1149</v>
       </c>
+      <c r="R166" t="b">
+        <v>0</v>
+      </c>
+      <c r="S166" t="inlineStr">
+        <is>
+          <t>Away=1.50 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="167">
-      <c r="A167" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A167" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
@@ -13284,12 +14286,18 @@
       <c r="Q167" t="n">
         <v>0.1379</v>
       </c>
+      <c r="R167" t="b">
+        <v>0</v>
+      </c>
+      <c r="S167" t="inlineStr">
+        <is>
+          <t>Away=1.47 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A168" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
@@ -13361,12 +14369,18 @@
       <c r="Q168" t="n">
         <v>0.1723</v>
       </c>
+      <c r="R168" t="b">
+        <v>1</v>
+      </c>
+      <c r="S168" t="inlineStr">
+        <is>
+          <t>Away=1.62 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="169">
-      <c r="A169" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
+      <c r="A169" s="2" t="n">
+        <v>46264</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
@@ -13438,12 +14452,18 @@
       <c r="Q169" t="n">
         <v>0.1122</v>
       </c>
+      <c r="R169" t="b">
+        <v>0</v>
+      </c>
+      <c r="S169" t="inlineStr">
+        <is>
+          <t>Away=1.44 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="170">
-      <c r="A170" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
+      <c r="A170" s="2" t="n">
+        <v>46265</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
@@ -13515,12 +14535,18 @@
       <c r="Q170" t="n">
         <v>-1</v>
       </c>
+      <c r="R170" t="b">
+        <v>0</v>
+      </c>
+      <c r="S170" t="inlineStr">
+        <is>
+          <t>Over3.5=2.26 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="171">
-      <c r="A171" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
+      <c r="A171" s="2" t="n">
+        <v>46265</v>
       </c>
       <c r="B171" t="inlineStr">
         <is>
@@ -13592,12 +14618,18 @@
       <c r="Q171" t="n">
         <v>0.193</v>
       </c>
+      <c r="R171" t="b">
+        <v>0</v>
+      </c>
+      <c r="S171" t="inlineStr">
+        <is>
+          <t>Over3.5=2.28 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
+      <c r="A172" s="2" t="n">
+        <v>46265</v>
       </c>
       <c r="B172" t="inlineStr">
         <is>
@@ -13669,12 +14701,18 @@
       <c r="Q172" t="n">
         <v>0.2144</v>
       </c>
+      <c r="R172" t="b">
+        <v>1</v>
+      </c>
+      <c r="S172" t="inlineStr">
+        <is>
+          <t>Over3.5=3.15 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
+      <c r="A173" s="2" t="n">
+        <v>46265</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
@@ -13746,12 +14784,18 @@
       <c r="Q173" t="n">
         <v>0.193</v>
       </c>
+      <c r="R173" t="b">
+        <v>1</v>
+      </c>
+      <c r="S173" t="inlineStr">
+        <is>
+          <t>Away=1.64 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
+      <c r="A174" s="2" t="n">
+        <v>46265</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
@@ -13823,12 +14867,18 @@
       <c r="Q174" t="n">
         <v>0.1419</v>
       </c>
+      <c r="R174" t="b">
+        <v>1</v>
+      </c>
+      <c r="S174" t="inlineStr">
+        <is>
+          <t>Away=1.62 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
+      <c r="A175" s="2" t="n">
+        <v>46265</v>
       </c>
       <c r="B175" t="inlineStr">
         <is>
@@ -13900,12 +14950,18 @@
       <c r="Q175" t="n">
         <v>0.1608</v>
       </c>
+      <c r="R175" t="b">
+        <v>0</v>
+      </c>
+      <c r="S175" t="inlineStr">
+        <is>
+          <t>Away=1.47 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
+      <c r="A176" s="2" t="n">
+        <v>46265</v>
       </c>
       <c r="B176" t="inlineStr">
         <is>
@@ -13977,12 +15033,18 @@
       <c r="Q176" t="n">
         <v>0.1723</v>
       </c>
+      <c r="R176" t="b">
+        <v>1</v>
+      </c>
+      <c r="S176" t="inlineStr">
+        <is>
+          <t>Away=1.65 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
+      <c r="A177" s="2" t="n">
+        <v>46265</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
@@ -14054,12 +15116,18 @@
       <c r="Q177" t="n">
         <v>0.1304</v>
       </c>
+      <c r="R177" t="b">
+        <v>0</v>
+      </c>
+      <c r="S177" t="inlineStr">
+        <is>
+          <t>Away=1.50 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
+      <c r="A178" s="2" t="n">
+        <v>46265</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
@@ -14131,12 +15199,18 @@
       <c r="Q178" t="n">
         <v>0.1556</v>
       </c>
+      <c r="R178" t="b">
+        <v>1</v>
+      </c>
+      <c r="S178" t="inlineStr">
+        <is>
+          <t>Away=1.54 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
+      <c r="A179" s="2" t="n">
+        <v>46265</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
@@ -14208,12 +15282,18 @@
       <c r="Q179" t="n">
         <v>0.0551</v>
       </c>
+      <c r="R179" t="b">
+        <v>1</v>
+      </c>
+      <c r="S179" t="inlineStr">
+        <is>
+          <t>Under &lt;= 1.50</t>
+        </is>
+      </c>
     </row>
     <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
+      <c r="A180" s="2" t="n">
+        <v>46266</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
@@ -14285,12 +15365,18 @@
       <c r="Q180" t="n">
         <v>0.2298</v>
       </c>
+      <c r="R180" t="b">
+        <v>1</v>
+      </c>
+      <c r="S180" t="inlineStr">
+        <is>
+          <t>Over3.5=3.50 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
+      <c r="A181" s="2" t="n">
+        <v>46266</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
@@ -14362,12 +15448,18 @@
       <c r="Q181" t="n">
         <v>0.1237</v>
       </c>
+      <c r="R181" t="b">
+        <v>1</v>
+      </c>
+      <c r="S181" t="inlineStr">
+        <is>
+          <t>Over3.5=2.56 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
+      <c r="A182" s="2" t="n">
+        <v>46266</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
@@ -14439,12 +15531,18 @@
       <c r="Q182" t="n">
         <v>0.1508</v>
       </c>
+      <c r="R182" t="b">
+        <v>0</v>
+      </c>
+      <c r="S182" t="inlineStr">
+        <is>
+          <t>Away=1.53 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
+      <c r="A183" s="2" t="n">
+        <v>46266</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
@@ -14516,12 +15614,18 @@
       <c r="Q183" t="n">
         <v>0.1508</v>
       </c>
+      <c r="R183" t="b">
+        <v>0</v>
+      </c>
+      <c r="S183" t="inlineStr">
+        <is>
+          <t>Away=1.45 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
+      <c r="A184" s="2" t="n">
+        <v>46266</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
@@ -14593,12 +15697,18 @@
       <c r="Q184" t="n">
         <v>0.2244</v>
       </c>
+      <c r="R184" t="b">
+        <v>1</v>
+      </c>
+      <c r="S184" t="inlineStr">
+        <is>
+          <t>Away=1.63 ([1.54, 1.65])</t>
+        </is>
+      </c>
     </row>
     <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
+      <c r="A185" s="2" t="n">
+        <v>46267</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
@@ -14670,12 +15780,18 @@
       <c r="Q185" t="n">
         <v>0.1556</v>
       </c>
+      <c r="R185" t="b">
+        <v>1</v>
+      </c>
+      <c r="S185" t="inlineStr">
+        <is>
+          <t>Over3.5=2.62 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
+      <c r="A186" s="2" t="n">
+        <v>46267</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -14747,12 +15863,18 @@
       <c r="Q186" t="n">
         <v>0.1787</v>
       </c>
+      <c r="R186" t="b">
+        <v>1</v>
+      </c>
+      <c r="S186" t="inlineStr">
+        <is>
+          <t>Over3.5=2.94 (&gt;=2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
+      <c r="A187" s="2" t="n">
+        <v>46267</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
@@ -14824,12 +15946,18 @@
       <c r="Q187" t="n">
         <v>0.1556</v>
       </c>
+      <c r="R187" t="b">
+        <v>0</v>
+      </c>
+      <c r="S187" t="inlineStr">
+        <is>
+          <t>Over3.5=2.12 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="188">
-      <c r="A188" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
+      <c r="A188" s="2" t="n">
+        <v>46267</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
@@ -14901,12 +16029,18 @@
       <c r="Q188" t="n">
         <v>0.1462</v>
       </c>
+      <c r="R188" t="b">
+        <v>0</v>
+      </c>
+      <c r="S188" t="inlineStr">
+        <is>
+          <t>Over3.5=2.46 (&lt;2.54)</t>
+        </is>
+      </c>
     </row>
     <row r="189">
-      <c r="A189" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
+      <c r="A189" s="2" t="n">
+        <v>46267</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
@@ -14978,12 +16112,18 @@
       <c r="Q189" t="n">
         <v>0.1072</v>
       </c>
+      <c r="R189" t="b">
+        <v>0</v>
+      </c>
+      <c r="S189" t="inlineStr">
+        <is>
+          <t>Away=1.44 (fora da faixa)</t>
+        </is>
+      </c>
     </row>
     <row r="190">
-      <c r="A190" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
+      <c r="A190" s="2" t="n">
+        <v>46267</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
@@ -15054,6 +16194,14 @@
       </c>
       <c r="Q190" t="n">
         <v>0.1969</v>
+      </c>
+      <c r="R190" t="b">
+        <v>1</v>
+      </c>
+      <c r="S190" t="inlineStr">
+        <is>
+          <t>Away=1.64 ([1.54, 1.65])</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>